<commit_message>
Add Shanghai, Nanchang, Shenyang G-train and Hong Kong Value variants
- Shanghai: Sleeper / Spring nonstop / Train (no sleeper), Trip.com + 12306 fares
- Nanchang: Sleeper (Air China + Z111) / Comfort / Fly in, JXNU Yaohu hotels
- Shenyang: G-train versions of Comfort and Budget (no sleeper trains)
- Hong Kong: Value variant, refreshed hotel and Trip.com flight prices
- Compare sheet: 15 plans, new picks and notes; fares workbook: 10 Oct sheet
- details.md: Trip.com flights in the browser, CTO sale dates, results
- q12306.py: Q12306_INSECURE for Windows

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ICPC_flight_fares_30Sep2026.xlsx
+++ b/ICPC_flight_fares_30Sep2026.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Connector notes" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Trains &amp; hotels" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="12306 &amp; ChinaTicketOnline" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="10 Oct – Dec &amp; Jan checks" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -193,7 +194,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -385,6 +386,9 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5316,7 +5320,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="25" t="inlineStr">
         <is>
           <t>USD → CNY (from MNT rates 3598 / 536)</t>
         </is>
@@ -5371,4 +5375,876 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" style="26" min="1" max="1"/>
+    <col width="11" customWidth="1" style="26" min="2" max="2"/>
+    <col width="44" customWidth="1" style="26" min="3" max="3"/>
+    <col width="22" customWidth="1" style="26" min="4" max="4"/>
+    <col width="20" customWidth="1" style="26" min="5" max="5"/>
+    <col width="30" customWidth="1" style="26" min="6" max="6"/>
+    <col width="34" customWidth="1" style="26" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="62" t="inlineStr">
+        <is>
+          <t>Shanghai, Nanchang, Shenyang and Hong Kong checks (10 Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1" s="26">
+      <c r="A2" s="60" t="inlineStr">
+        <is>
+          <t>Flights: Trip.com in the built-in browser (open the m/flights URL in a fronted tab and wait ~40 s; background tabs do not finish loading) and SlickTrip. Trains: 12306 fares for the 20 Oct train (fares are fixed), ChinaTicketOnline for timetables and sale dates of the real plan dates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="69" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B4" s="69" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C4" s="69" t="inlineStr">
+        <is>
+          <t>Option</t>
+        </is>
+      </c>
+      <c r="D4" s="69" t="inlineStr">
+        <is>
+          <t>Trip.com (USD / CNY)</t>
+        </is>
+      </c>
+      <c r="E4" s="69" t="inlineStr">
+        <is>
+          <t>SlickTrip (USD)</t>
+        </is>
+      </c>
+      <c r="F4" s="69" t="inlineStr">
+        <is>
+          <t>12306 / CTO</t>
+        </is>
+      </c>
+      <c r="G4" s="69" t="inlineStr">
+        <is>
+          <t>Used in</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="60" t="inlineStr">
+        <is>
+          <t>Flight UB → Beijing</t>
+        </is>
+      </c>
+      <c r="B5" s="60" t="inlineStr">
+        <is>
+          <t>17 Dec</t>
+        </is>
+      </c>
+      <c r="C5" s="60" t="inlineStr">
+        <is>
+          <t>Air China CA956 16:10–18:20</t>
+        </is>
+      </c>
+      <c r="D5" s="60" t="inlineStr">
+        <is>
+          <t>$157</t>
+        </is>
+      </c>
+      <c r="E5" s="60" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F5" s="60" t="inlineStr"/>
+      <c r="G5" s="60" t="inlineStr">
+        <is>
+          <t>Nanchang – Sleeper</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="60" t="inlineStr">
+        <is>
+          <t>Flight UB → Beijing</t>
+        </is>
+      </c>
+      <c r="B6" s="60" t="inlineStr">
+        <is>
+          <t>17 Dec</t>
+        </is>
+      </c>
+      <c r="C6" s="60" t="inlineStr">
+        <is>
+          <t>MIAT OM223 07:30–09:45</t>
+        </is>
+      </c>
+      <c r="D6" s="60" t="inlineStr">
+        <is>
+          <t>$193</t>
+        </is>
+      </c>
+      <c r="E6" s="60" t="inlineStr">
+        <is>
+          <t>$196</t>
+        </is>
+      </c>
+      <c r="F6" s="60" t="inlineStr"/>
+      <c r="G6" s="60" t="inlineStr">
+        <is>
+          <t>Nanchang – Comfort</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="60" t="inlineStr">
+        <is>
+          <t>Flight UB → Beijing</t>
+        </is>
+      </c>
+      <c r="B7" s="60" t="inlineStr">
+        <is>
+          <t>17 Dec</t>
+        </is>
+      </c>
+      <c r="C7" s="60" t="inlineStr">
+        <is>
+          <t>Air China CA902 11:50–13:55</t>
+        </is>
+      </c>
+      <c r="D7" s="60" t="inlineStr">
+        <is>
+          <t>$363 ($354 student)</t>
+        </is>
+      </c>
+      <c r="E7" s="60" t="inlineStr">
+        <is>
+          <t>$356 through to KHN</t>
+        </is>
+      </c>
+      <c r="F7" s="60" t="inlineStr"/>
+      <c r="G7" s="60" t="inlineStr">
+        <is>
+          <t>Nanchang – Fly in</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="60" t="inlineStr">
+        <is>
+          <t>Flight Beijing → UB</t>
+        </is>
+      </c>
+      <c r="B8" s="60" t="inlineStr">
+        <is>
+          <t>21 Dec</t>
+        </is>
+      </c>
+      <c r="C8" s="60" t="inlineStr">
+        <is>
+          <t>Air China CA955 12:55–15:05 (08:25 also $172)</t>
+        </is>
+      </c>
+      <c r="D8" s="60" t="inlineStr">
+        <is>
+          <t>$172</t>
+        </is>
+      </c>
+      <c r="E8" s="60" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F8" s="60" t="inlineStr"/>
+      <c r="G8" s="60" t="inlineStr">
+        <is>
+          <t>Nanchang (all)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="60" t="inlineStr">
+        <is>
+          <t>Flight Beijing → UB</t>
+        </is>
+      </c>
+      <c r="B9" s="60" t="inlineStr">
+        <is>
+          <t>21 Dec</t>
+        </is>
+      </c>
+      <c r="C9" s="60" t="inlineStr">
+        <is>
+          <t>MIAT OM224 11:30–13:50</t>
+        </is>
+      </c>
+      <c r="D9" s="60" t="inlineStr">
+        <is>
+          <t>$193</t>
+        </is>
+      </c>
+      <c r="E9" s="60" t="inlineStr">
+        <is>
+          <t>$224</t>
+        </is>
+      </c>
+      <c r="F9" s="60" t="inlineStr"/>
+      <c r="G9" s="60" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="60" t="inlineStr">
+        <is>
+          <t>Flight UB → Beijing</t>
+        </is>
+      </c>
+      <c r="B10" s="60" t="inlineStr">
+        <is>
+          <t>3 Dec</t>
+        </is>
+      </c>
+      <c r="C10" s="60" t="inlineStr">
+        <is>
+          <t>MIAT OM223 07:30–09:45</t>
+        </is>
+      </c>
+      <c r="D10" s="60" t="inlineStr">
+        <is>
+          <t>$151</t>
+        </is>
+      </c>
+      <c r="E10" s="60" t="inlineStr">
+        <is>
+          <t>$154</t>
+        </is>
+      </c>
+      <c r="F10" s="60" t="inlineStr"/>
+      <c r="G10" s="60" t="inlineStr">
+        <is>
+          <t>Shanghai (A, C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="60" t="inlineStr">
+        <is>
+          <t>Flight UB → Beijing</t>
+        </is>
+      </c>
+      <c r="B11" s="60" t="inlineStr">
+        <is>
+          <t>3 Dec</t>
+        </is>
+      </c>
+      <c r="C11" s="60" t="inlineStr">
+        <is>
+          <t>Air China 11:50–13:55</t>
+        </is>
+      </c>
+      <c r="D11" s="60" t="inlineStr">
+        <is>
+          <t>$200</t>
+        </is>
+      </c>
+      <c r="E11" s="60" t="inlineStr"/>
+      <c r="F11" s="60" t="inlineStr"/>
+      <c r="G11" s="60" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="60" t="inlineStr">
+        <is>
+          <t>Flight Beijing → UB</t>
+        </is>
+      </c>
+      <c r="B12" s="60" t="inlineStr">
+        <is>
+          <t>7 Dec</t>
+        </is>
+      </c>
+      <c r="C12" s="60" t="inlineStr">
+        <is>
+          <t>Air China CA955 12:55–15:05 (08:25 also $172)</t>
+        </is>
+      </c>
+      <c r="D12" s="60" t="inlineStr">
+        <is>
+          <t>$172</t>
+        </is>
+      </c>
+      <c r="E12" s="60" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F12" s="60" t="inlineStr"/>
+      <c r="G12" s="60" t="inlineStr">
+        <is>
+          <t>Shanghai (A, C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="60" t="inlineStr">
+        <is>
+          <t>Flight Beijing → UB</t>
+        </is>
+      </c>
+      <c r="B13" s="60" t="inlineStr">
+        <is>
+          <t>7 Dec</t>
+        </is>
+      </c>
+      <c r="C13" s="60" t="inlineStr">
+        <is>
+          <t>MIAT OM224 11:30–13:50</t>
+        </is>
+      </c>
+      <c r="D13" s="60" t="inlineStr">
+        <is>
+          <t>$193</t>
+        </is>
+      </c>
+      <c r="E13" s="60" t="inlineStr">
+        <is>
+          <t>$197</t>
+        </is>
+      </c>
+      <c r="F13" s="60" t="inlineStr"/>
+      <c r="G13" s="60" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="60" t="inlineStr">
+        <is>
+          <t>Flight UB → Shanghai</t>
+        </is>
+      </c>
+      <c r="B14" s="60" t="inlineStr">
+        <is>
+          <t>1 Dec</t>
+        </is>
+      </c>
+      <c r="C14" s="60" t="inlineStr">
+        <is>
+          <t>Spring 9C6520 13:00–17:00 PVG</t>
+        </is>
+      </c>
+      <c r="D14" s="60" t="inlineStr">
+        <is>
+          <t>$173</t>
+        </is>
+      </c>
+      <c r="E14" s="60" t="inlineStr">
+        <is>
+          <t>$164</t>
+        </is>
+      </c>
+      <c r="F14" s="60" t="inlineStr"/>
+      <c r="G14" s="60" t="inlineStr">
+        <is>
+          <t>Shanghai – Spring nonstop</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="60" t="inlineStr">
+        <is>
+          <t>Flight Shanghai → UB</t>
+        </is>
+      </c>
+      <c r="B15" s="60" t="inlineStr">
+        <is>
+          <t>8 Dec</t>
+        </is>
+      </c>
+      <c r="C15" s="60" t="inlineStr">
+        <is>
+          <t>Spring 9C6519 08:00–12:00 PVG</t>
+        </is>
+      </c>
+      <c r="D15" s="60" t="inlineStr">
+        <is>
+          <t>$159</t>
+        </is>
+      </c>
+      <c r="E15" s="60" t="inlineStr">
+        <is>
+          <t>$153</t>
+        </is>
+      </c>
+      <c r="F15" s="60" t="inlineStr"/>
+      <c r="G15" s="60" t="inlineStr">
+        <is>
+          <t>Shanghai – Spring nonstop</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="60" t="inlineStr">
+        <is>
+          <t>Flight UB ⇄ Hong Kong</t>
+        </is>
+      </c>
+      <c r="B16" s="60" t="inlineStr">
+        <is>
+          <t>8–11 Jan</t>
+        </is>
+      </c>
+      <c r="C16" s="60" t="inlineStr">
+        <is>
+          <t>MIAT nonstop round trip</t>
+        </is>
+      </c>
+      <c r="D16" s="60" t="inlineStr">
+        <is>
+          <t>$586 (30 Sep: $583)</t>
+        </is>
+      </c>
+      <c r="E16" s="60" t="inlineStr">
+        <is>
+          <t>$593</t>
+        </is>
+      </c>
+      <c r="F16" s="60" t="inlineStr"/>
+      <c r="G16" s="60" t="inlineStr">
+        <is>
+          <t>Hong Kong (all)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="60" t="inlineStr">
+        <is>
+          <t>Flight Hohhot → HKG/SZX</t>
+        </is>
+      </c>
+      <c r="B17" s="60" t="inlineStr">
+        <is>
+          <t>8 Jan</t>
+        </is>
+      </c>
+      <c r="C17" s="60" t="inlineStr">
+        <is>
+          <t>Shenzhen Airlines HET → SZX 15:45</t>
+        </is>
+      </c>
+      <c r="D17" s="60" t="inlineStr"/>
+      <c r="E17" s="60" t="inlineStr">
+        <is>
+          <t>$214</t>
+        </is>
+      </c>
+      <c r="F17" s="60" t="inlineStr"/>
+      <c r="G17" s="60" t="inlineStr">
+        <is>
+          <t>Not used (Aero Mongolia ¥892 + $214 &gt; $293)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="60" t="inlineStr">
+        <is>
+          <t>Flight Beijing → HKG</t>
+        </is>
+      </c>
+      <c r="B18" s="60" t="inlineStr">
+        <is>
+          <t>8 Jan</t>
+        </is>
+      </c>
+      <c r="C18" s="60" t="inlineStr">
+        <is>
+          <t>Cathay CX345 07:30</t>
+        </is>
+      </c>
+      <c r="D18" s="60" t="inlineStr"/>
+      <c r="E18" s="60" t="inlineStr">
+        <is>
+          <t>$206</t>
+        </is>
+      </c>
+      <c r="F18" s="60" t="inlineStr"/>
+      <c r="G18" s="60" t="inlineStr">
+        <is>
+          <t>Not used (MIAT $150–196 + $206)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="60" t="inlineStr">
+        <is>
+          <t>Train Beijing Fengtai → Nanchang</t>
+        </is>
+      </c>
+      <c r="B19" s="60" t="inlineStr">
+        <is>
+          <t>17 Dec</t>
+        </is>
+      </c>
+      <c r="C19" s="60" t="inlineStr">
+        <is>
+          <t>Z111 23:06 → 11:52, hard sleeper</t>
+        </is>
+      </c>
+      <c r="D19" s="60" t="inlineStr"/>
+      <c r="E19" s="60" t="inlineStr"/>
+      <c r="F19" s="60" t="inlineStr">
+        <is>
+          <t>12306 ¥296.5 / CTO $50+9.5</t>
+        </is>
+      </c>
+      <c r="G19" s="60" t="inlineStr">
+        <is>
+          <t>Nanchang – Sleeper</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="60" t="inlineStr">
+        <is>
+          <t>Train Beijing Fengtai → Nanchang</t>
+        </is>
+      </c>
+      <c r="B20" s="60" t="inlineStr">
+        <is>
+          <t>17 Dec</t>
+        </is>
+      </c>
+      <c r="C20" s="60" t="inlineStr">
+        <is>
+          <t>D135 19:48 → 07:49, 2nd-class sleeper</t>
+        </is>
+      </c>
+      <c r="D20" s="60" t="inlineStr"/>
+      <c r="E20" s="60" t="inlineStr"/>
+      <c r="F20" s="60" t="inlineStr">
+        <is>
+          <t>12306 ¥382 / CTO $69+10.5</t>
+        </is>
+      </c>
+      <c r="G20" s="60" t="inlineStr">
+        <is>
+          <t>Backup (MIAT 07:30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="60" t="inlineStr">
+        <is>
+          <t>Train Beijing West → Nanchang West</t>
+        </is>
+      </c>
+      <c r="B21" s="60" t="inlineStr">
+        <is>
+          <t>17 Dec</t>
+        </is>
+      </c>
+      <c r="C21" s="60" t="inlineStr">
+        <is>
+          <t>G335 12:00 → 17:52</t>
+        </is>
+      </c>
+      <c r="D21" s="60" t="inlineStr"/>
+      <c r="E21" s="60" t="inlineStr"/>
+      <c r="F21" s="60" t="inlineStr">
+        <is>
+          <t>12306 ¥745 / CTO $118+12</t>
+        </is>
+      </c>
+      <c r="G21" s="60" t="inlineStr">
+        <is>
+          <t>Nanchang – Comfort</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="60" t="inlineStr">
+        <is>
+          <t>Train Nanchang → Beijing Fengtai</t>
+        </is>
+      </c>
+      <c r="B22" s="60" t="inlineStr">
+        <is>
+          <t>20 Dec</t>
+        </is>
+      </c>
+      <c r="C22" s="60" t="inlineStr">
+        <is>
+          <t>D136 19:22 → 07:31, 2nd-class sleeper</t>
+        </is>
+      </c>
+      <c r="D22" s="60" t="inlineStr"/>
+      <c r="E22" s="60" t="inlineStr"/>
+      <c r="F22" s="60" t="inlineStr">
+        <is>
+          <t>12306 ¥382 / CTO $69+10.5</t>
+        </is>
+      </c>
+      <c r="G22" s="60" t="inlineStr">
+        <is>
+          <t>Nanchang (all)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="60" t="inlineStr">
+        <is>
+          <t>Train Beijing South → Shanghai</t>
+        </is>
+      </c>
+      <c r="B23" s="60" t="inlineStr">
+        <is>
+          <t>3 Dec</t>
+        </is>
+      </c>
+      <c r="C23" s="60" t="inlineStr">
+        <is>
+          <t>G17 13:00 → 17:35</t>
+        </is>
+      </c>
+      <c r="D23" s="60" t="inlineStr"/>
+      <c r="E23" s="60" t="inlineStr"/>
+      <c r="F23" s="60" t="inlineStr">
+        <is>
+          <t>12306 ¥667 / CTO $124+15</t>
+        </is>
+      </c>
+      <c r="G23" s="60" t="inlineStr">
+        <is>
+          <t>Shanghai (all)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="60" t="inlineStr">
+        <is>
+          <t>Train Shanghai → Beijing Fengtai</t>
+        </is>
+      </c>
+      <c r="B24" s="60" t="inlineStr">
+        <is>
+          <t>6 Dec</t>
+        </is>
+      </c>
+      <c r="C24" s="60" t="inlineStr">
+        <is>
+          <t>D8 19:08 → 06:58/07:17, 2nd-class sleeper</t>
+        </is>
+      </c>
+      <c r="D24" s="60" t="inlineStr"/>
+      <c r="E24" s="60" t="inlineStr"/>
+      <c r="F24" s="60" t="inlineStr">
+        <is>
+          <t>12306 ¥440 / CTO $97+12 (¥625)</t>
+        </is>
+      </c>
+      <c r="G24" s="60" t="inlineStr">
+        <is>
+          <t>Shanghai – Sleeper</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="60" t="inlineStr">
+        <is>
+          <t>Train Hongqiao → Beijing South</t>
+        </is>
+      </c>
+      <c r="B25" s="60" t="inlineStr">
+        <is>
+          <t>6 Dec</t>
+        </is>
+      </c>
+      <c r="C25" s="60" t="inlineStr">
+        <is>
+          <t>G32 19:25 → 23:49</t>
+        </is>
+      </c>
+      <c r="D25" s="60" t="inlineStr"/>
+      <c r="E25" s="60" t="inlineStr"/>
+      <c r="F25" s="60" t="inlineStr">
+        <is>
+          <t>12306 ¥598 / CTO $123+15</t>
+        </is>
+      </c>
+      <c r="G25" s="60" t="inlineStr">
+        <is>
+          <t>Shanghai – Train (no sleeper)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="60" t="inlineStr">
+        <is>
+          <t>Train Beijing Chaoyang → Shenyang N.</t>
+        </is>
+      </c>
+      <c r="B26" s="60" t="inlineStr">
+        <is>
+          <t>12 Nov</t>
+        </is>
+      </c>
+      <c r="C26" s="60" t="inlineStr">
+        <is>
+          <t>G149 12:19 → 14:48</t>
+        </is>
+      </c>
+      <c r="D26" s="60" t="inlineStr"/>
+      <c r="E26" s="60" t="inlineStr"/>
+      <c r="F26" s="60" t="inlineStr">
+        <is>
+          <t>12306 ¥369</t>
+        </is>
+      </c>
+      <c r="G26" s="60" t="inlineStr">
+        <is>
+          <t>Shenyang – Comfort (G-train)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="60" t="inlineStr">
+        <is>
+          <t>Train Beijing Chaoyang → Shenyang N.</t>
+        </is>
+      </c>
+      <c r="B27" s="60" t="inlineStr">
+        <is>
+          <t>14 Nov</t>
+        </is>
+      </c>
+      <c r="C27" s="60" t="inlineStr">
+        <is>
+          <t>G101 08:00 → 10:29</t>
+        </is>
+      </c>
+      <c r="D27" s="60" t="inlineStr"/>
+      <c r="E27" s="60" t="inlineStr"/>
+      <c r="F27" s="60" t="inlineStr">
+        <is>
+          <t>12306 ¥355</t>
+        </is>
+      </c>
+      <c r="G27" s="60" t="inlineStr">
+        <is>
+          <t>Shenyang – Budget (G-train)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="60" t="inlineStr">
+        <is>
+          <t>Train Shenyang N. → Beijing Chaoyang</t>
+        </is>
+      </c>
+      <c r="B28" s="60" t="inlineStr">
+        <is>
+          <t>15 Nov</t>
+        </is>
+      </c>
+      <c r="C28" s="60" t="inlineStr">
+        <is>
+          <t>G142 19:51 → 22:30</t>
+        </is>
+      </c>
+      <c r="D28" s="60" t="inlineStr"/>
+      <c r="E28" s="60" t="inlineStr"/>
+      <c r="F28" s="60" t="inlineStr">
+        <is>
+          <t>12306 ¥268</t>
+        </is>
+      </c>
+      <c r="G28" s="60" t="inlineStr">
+        <is>
+          <t>Shenyang (G-train)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="68" t="inlineStr">
+        <is>
+          <t>Sale dates (Beijing time; train on date D opens D − 14 days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Z111 / D135 / G335, 17 Dec</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>3 Dec 08:00 (Fengtai / Beijing West)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>D136, 20 Dec</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>6 Dec 09:45 (Nanchang station; Nanjing is 08:15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>G17, 3 Dec</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>19 Nov 12:45 (Beijing South)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>D8 / G32, 6 Dec</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>22 Nov 14:45 / 13:45 (Shanghai / Hongqiao)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>D17 Beijing → Hangzhou, 25 Jan</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>11 Jan 10:00 (Beijing)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:G2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Shenyang: budget hotels around NEU grouped by walk / metro / taxi
New sheet "Shenyang hotels by distance" in ICPC_flight_fares_30Sep2026.xlsx:
Tripadvisor (Trip.com/Agoda/Booking prices) and Booking.com results for
12-15 Nov, 2 rooms x 3 nights, with distance to NEU, nearest metro and
estimated metro / taxi time and fare. Notes Metro Line 3 (Sanhaojie,
~0.5 km from campus, opened 30 Jun 2026) and the commute-cost check.
details.md records the findings and the tool behaviour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018GZDCacqRiEe328BLfJXxj
</commit_message>
<xml_diff>
--- a/ICPC_flight_fares_30Sep2026.xlsx
+++ b/ICPC_flight_fares_30Sep2026.xlsx
@@ -1,17 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Flight fares" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Connector notes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Trains &amp; hotels" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="12306 &amp; ChinaTicketOnline" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="10 Oct – Dec &amp; Jan checks" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flight fares" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connector notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trains &amp; hotels" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12306 &amp; ChinaTicketOnline" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Oct – Dec &amp; Jan checks" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shenyang hotels by distance" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -20,11 +21,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
     <numFmt numFmtId="165" formatCode="#,##0&quot; ₮&quot;;\(#,##0&quot; ₮)&quot;;\-"/>
+    <numFmt numFmtId="166" formatCode="#,##0&quot; ₮&quot;"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -122,8 +124,27 @@
     <font>
       <color rgb="000000FF"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF0000FF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -157,6 +178,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -194,7 +230,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -389,6 +425,35 @@
     <xf numFmtId="0" fontId="14" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6182,60 +6247,60 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="25" t="inlineStr">
         <is>
           <t>Z111 / D135 / G335, 17 Dec</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="25" t="inlineStr">
         <is>
           <t>3 Dec 08:00 (Fengtai / Beijing West)</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="25" t="inlineStr">
         <is>
           <t>D136, 20 Dec</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="25" t="inlineStr">
         <is>
           <t>6 Dec 09:45 (Nanchang station; Nanjing is 08:15)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="25" t="inlineStr">
         <is>
           <t>G17, 3 Dec</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="25" t="inlineStr">
         <is>
           <t>19 Nov 12:45 (Beijing South)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="25" t="inlineStr">
         <is>
           <t>D8 / G32, 6 Dec</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="25" t="inlineStr">
         <is>
           <t>22 Nov 14:45 / 13:45 (Shanghai / Hongqiao)</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="25" t="inlineStr">
         <is>
           <t>D17 Beijing → Hangzhou, 25 Jan</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="25" t="inlineStr">
         <is>
           <t>11 Jan 10:00 (Beijing)</t>
         </is>
@@ -6247,4 +6312,2477 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L67"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" style="26" min="1" max="1"/>
+    <col width="44" customWidth="1" style="26" min="2" max="2"/>
+    <col width="11" customWidth="1" style="26" min="3" max="3"/>
+    <col width="8" customWidth="1" style="26" min="4" max="4"/>
+    <col width="30" customWidth="1" style="26" min="5" max="5"/>
+    <col width="26" customWidth="1" style="26" min="6" max="6"/>
+    <col width="16" customWidth="1" style="26" min="7" max="7"/>
+    <col width="14" customWidth="1" style="26" min="8" max="8"/>
+    <col width="9" customWidth="1" style="26" min="9" max="9"/>
+    <col width="13" customWidth="1" style="26" min="10" max="10"/>
+    <col width="22" customWidth="1" style="26" min="11" max="11"/>
+    <col width="60" customWidth="1" style="26" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="70" t="inlineStr">
+        <is>
+          <t>Budget hotels around NEU Nanhu campus, Shenyang – by how you reach campus (searched 22 Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="92" customHeight="1" s="26">
+      <c r="A2" s="71" t="inlineStr">
+        <is>
+          <t>Stay 12–15 Nov 2026 (3 nights). Price = 2 rooms × 3 nights, the team price for 3 or 4 people (Tripadvisor search with 4 adults / 2 rooms; its partner prices exclude ~$1–3 tax). Distances are straight-line from the Trip.com NEU landmark (41.7655, 123.4182, campus centre); the contest building is not confirmed, so allow ±0.5 km. Nearest metro to NEU: Line 3 Sanhaojie station on Wenhua Road (~0.5 km; Line 3 east section opened 30 Jun 2026). Times are estimates: walk 75 m/min × 1.25 detour; metro = walk + 4 min wait + 2.3 min per stop + 5 min per change + 9 min walk from Sanhaojie; taxi = 1.35 × straight-line at 22 km/h + 3 min, fare ¥9 for 3 km + ¥2/km (2025 tariff per taxi-rechner.de, not confirmed officially). Metro fares start at ¥2 per person. Cheapest rates may be double-bed rooms; small independent hotels may not register foreign guests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="72" t="inlineStr">
+        <is>
+          <t>USD → MNT</t>
+        </is>
+      </c>
+      <c r="B3" s="73" t="n">
+        <v>3598</v>
+      </c>
+      <c r="C3" s="72" t="inlineStr">
+        <is>
+          <t>CNY → MNT</t>
+        </is>
+      </c>
+      <c r="D3" s="73" t="n">
+        <v>536</v>
+      </c>
+      <c r="E3" s="74" t="inlineStr">
+        <is>
+          <t>Same rates as Compare!B8:B9 in ICPC_Single_Contest_Plans.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="75" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="B5" s="75" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="C5" s="75" t="inlineStr">
+        <is>
+          <t>Distance to NEU (km)</t>
+        </is>
+      </c>
+      <c r="D5" s="75" t="inlineStr">
+        <is>
+          <t>Walk (min)</t>
+        </is>
+      </c>
+      <c r="E5" s="75" t="inlineStr">
+        <is>
+          <t>Nearest metro (walk km)</t>
+        </is>
+      </c>
+      <c r="F5" s="75" t="inlineStr">
+        <is>
+          <t>Metro to NEU (min)</t>
+        </is>
+      </c>
+      <c r="G5" s="75" t="inlineStr">
+        <is>
+          <t>Taxi to NEU (min / ¥ per car)</t>
+        </is>
+      </c>
+      <c r="H5" s="75" t="inlineStr">
+        <is>
+          <t>Team price (2 rooms × 3 nights)</t>
+        </is>
+      </c>
+      <c r="I5" s="75" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="J5" s="75" t="inlineStr">
+        <is>
+          <t>Total MNT</t>
+        </is>
+      </c>
+      <c r="K5" s="75" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="L5" s="75" t="inlineStr">
+        <is>
+          <t>Source / note</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="76" t="inlineStr">
+        <is>
+          <t>WALK – within ~1.5 km (≤ ~22 min on foot)</t>
+        </is>
+      </c>
+      <c r="B6" s="77" t="n"/>
+      <c r="C6" s="77" t="n"/>
+      <c r="D6" s="77" t="n"/>
+      <c r="E6" s="77" t="n"/>
+      <c r="F6" s="77" t="n"/>
+      <c r="G6" s="77" t="n"/>
+      <c r="H6" s="77" t="n"/>
+      <c r="I6" s="77" t="n"/>
+      <c r="J6" s="77" t="n"/>
+      <c r="K6" s="77" t="n"/>
+      <c r="L6" s="77" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="71" t="inlineStr">
+        <is>
+          <t>Walk</t>
+        </is>
+      </c>
+      <c r="B7" s="71" t="inlineStr">
+        <is>
+          <t>7 Days Inn Sanhao Street Liaozhan</t>
+        </is>
+      </c>
+      <c r="C7" s="78" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="D7" s="71" t="n">
+        <v>22</v>
+      </c>
+      <c r="E7" s="71" t="inlineStr">
+        <is>
+          <t>Gongye Zhanlanguan (L2/L3) (0.56)</t>
+        </is>
+      </c>
+      <c r="F7" s="71" t="inlineStr">
+        <is>
+          <t>– (walking is quicker)</t>
+        </is>
+      </c>
+      <c r="G7" s="71" t="inlineStr">
+        <is>
+          <t>8 / ¥9</t>
+        </is>
+      </c>
+      <c r="H7" s="79" t="n">
+        <v>95</v>
+      </c>
+      <c r="I7" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J7" s="80">
+        <f>H7*IF(I7="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K7" s="71" t="inlineStr">
+        <is>
+          <t>no reviews</t>
+        </is>
+      </c>
+      <c r="L7" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Booking.com, 22 Oct. chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="71" t="inlineStr">
+        <is>
+          <t>Walk</t>
+        </is>
+      </c>
+      <c r="B8" s="71" t="inlineStr">
+        <is>
+          <t>Home Inn Sanhao St / Shengjing 2nd Hospital</t>
+        </is>
+      </c>
+      <c r="C8" s="78" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="D8" s="71" t="n">
+        <v>19</v>
+      </c>
+      <c r="E8" s="71" t="inlineStr">
+        <is>
+          <t>Gongye Zhanlanguan (L2/L3) (0.19)</t>
+        </is>
+      </c>
+      <c r="F8" s="71" t="inlineStr">
+        <is>
+          <t>– (walking is quicker)</t>
+        </is>
+      </c>
+      <c r="G8" s="71" t="inlineStr">
+        <is>
+          <t>7 / ¥9</t>
+        </is>
+      </c>
+      <c r="H8" s="79" t="n">
+        <v>105</v>
+      </c>
+      <c r="I8" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J8" s="80">
+        <f>H8*IF(I8="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K8" s="71" t="inlineStr">
+        <is>
+          <t>no reviews</t>
+        </is>
+      </c>
+      <c r="L8" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Vio, 22 Oct. chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="71" t="inlineStr">
+        <is>
+          <t>Walk</t>
+        </is>
+      </c>
+      <c r="B9" s="71" t="inlineStr">
+        <is>
+          <t>7 Days Inn Shenyang Sanhao Street</t>
+        </is>
+      </c>
+      <c r="C9" s="78" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D9" s="71" t="n">
+        <v>12</v>
+      </c>
+      <c r="E9" s="71" t="inlineStr">
+        <is>
+          <t>Sanhaojie (L3) (0.91)</t>
+        </is>
+      </c>
+      <c r="F9" s="71" t="inlineStr">
+        <is>
+          <t>– (walking is quicker)</t>
+        </is>
+      </c>
+      <c r="G9" s="71" t="inlineStr">
+        <is>
+          <t>6 / ¥9</t>
+        </is>
+      </c>
+      <c r="H9" s="79" t="n">
+        <v>109</v>
+      </c>
+      <c r="I9" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J9" s="80">
+        <f>H9*IF(I9="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K9" s="71" t="inlineStr">
+        <is>
+          <t>TA 4.0 (1)</t>
+        </is>
+      </c>
+      <c r="L9" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Agoda, 22 Oct. chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="71" t="inlineStr">
+        <is>
+          <t>Walk</t>
+        </is>
+      </c>
+      <c r="B10" s="71" t="inlineStr">
+        <is>
+          <t>Jin Ke Hotel (Jinke)</t>
+        </is>
+      </c>
+      <c r="C10" s="78" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="D10" s="71" t="n">
+        <v>16</v>
+      </c>
+      <c r="E10" s="71" t="inlineStr">
+        <is>
+          <t>Gongye Zhanlanguan (L2/L3) (0.26)</t>
+        </is>
+      </c>
+      <c r="F10" s="71" t="inlineStr">
+        <is>
+          <t>– (walking is quicker)</t>
+        </is>
+      </c>
+      <c r="G10" s="71" t="inlineStr">
+        <is>
+          <t>6 / ¥9</t>
+        </is>
+      </c>
+      <c r="H10" s="79" t="n">
+        <v>146</v>
+      </c>
+      <c r="I10" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J10" s="80">
+        <f>H10*IF(I10="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K10" s="71" t="inlineStr">
+        <is>
+          <t>Trip.com 9.6; TA 3.4 (25)</t>
+        </is>
+      </c>
+      <c r="L10" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Trip.com, 22 Oct. Trip.com 22 Oct ¥1,044 for 2 rooms</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="71" t="inlineStr">
+        <is>
+          <t>Walk</t>
+        </is>
+      </c>
+      <c r="B11" s="71" t="inlineStr">
+        <is>
+          <t>Atour Hotel Youth Avenue Square (Booking)</t>
+        </is>
+      </c>
+      <c r="C11" s="78" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="D11" s="71" t="n">
+        <v>17</v>
+      </c>
+      <c r="E11" s="71" t="inlineStr">
+        <is>
+          <t>Sanhaojie (L3) (0.73)</t>
+        </is>
+      </c>
+      <c r="F11" s="71" t="inlineStr">
+        <is>
+          <t>– (walking is quicker)</t>
+        </is>
+      </c>
+      <c r="G11" s="71" t="inlineStr">
+        <is>
+          <t>7 / ¥9</t>
+        </is>
+      </c>
+      <c r="H11" s="79" t="n">
+        <v>1591</v>
+      </c>
+      <c r="I11" s="71" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J11" s="80">
+        <f>H11*IF(I11="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K11" s="71" t="inlineStr">
+        <is>
+          <t>new, no score</t>
+        </is>
+      </c>
+      <c r="L11" s="71" t="inlineStr">
+        <is>
+          <t>Booking.com, 22 Oct. 1 room for 3: ¥1,425</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="76" t="inlineStr">
+        <is>
+          <t>METRO – ≤ ~850 m from a station, Line 3 direct or one change from Line 2 (~25–35 min door to door)</t>
+        </is>
+      </c>
+      <c r="B12" s="77" t="n"/>
+      <c r="C12" s="77" t="n"/>
+      <c r="D12" s="77" t="n"/>
+      <c r="E12" s="77" t="n"/>
+      <c r="F12" s="77" t="n"/>
+      <c r="G12" s="77" t="n"/>
+      <c r="H12" s="77" t="n"/>
+      <c r="I12" s="77" t="n"/>
+      <c r="J12" s="77" t="n"/>
+      <c r="K12" s="77" t="n"/>
+      <c r="L12" s="77" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="71" t="inlineStr">
+        <is>
+          <t>Metro</t>
+        </is>
+      </c>
+      <c r="B13" s="71" t="inlineStr">
+        <is>
+          <t>Langrun Hotel</t>
+        </is>
+      </c>
+      <c r="C13" s="78" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="D13" s="71" t="n">
+        <v>36</v>
+      </c>
+      <c r="E13" s="71" t="inlineStr">
+        <is>
+          <t>Qingnian Gongyuan (L2) (0.22)</t>
+        </is>
+      </c>
+      <c r="F13" s="71" t="inlineStr">
+        <is>
+          <t>26 (L2&gt;L3, 2 stops, 1 change)</t>
+        </is>
+      </c>
+      <c r="G13" s="71" t="inlineStr">
+        <is>
+          <t>11 / ¥9</t>
+        </is>
+      </c>
+      <c r="H13" s="79" t="n">
+        <v>62</v>
+      </c>
+      <c r="I13" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J13" s="80">
+        <f>H13*IF(I13="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K13" s="71" t="inlineStr">
+        <is>
+          <t>no reviews</t>
+        </is>
+      </c>
+      <c r="L13" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Trip.com, 22 Oct. independent – check photos / foreign guests</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="71" t="inlineStr">
+        <is>
+          <t>Metro</t>
+        </is>
+      </c>
+      <c r="B14" s="71" t="inlineStr">
+        <is>
+          <t>Home Inn Youth Park Metro / TV Tower</t>
+        </is>
+      </c>
+      <c r="C14" s="78" t="n">
+        <v>2.87</v>
+      </c>
+      <c r="D14" s="71" t="n">
+        <v>48</v>
+      </c>
+      <c r="E14" s="71" t="inlineStr">
+        <is>
+          <t>Qingnian Gongyuan (L2) (0.80)</t>
+        </is>
+      </c>
+      <c r="F14" s="71" t="inlineStr">
+        <is>
+          <t>36 (L2&gt;L3, 2 stops, 1 change)</t>
+        </is>
+      </c>
+      <c r="G14" s="71" t="inlineStr">
+        <is>
+          <t>14 / ¥11</t>
+        </is>
+      </c>
+      <c r="H14" s="79" t="n">
+        <v>86</v>
+      </c>
+      <c r="I14" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J14" s="80">
+        <f>H14*IF(I14="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K14" s="71" t="inlineStr">
+        <is>
+          <t>no reviews</t>
+        </is>
+      </c>
+      <c r="L14" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Agoda, 22 Oct. chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="71" t="inlineStr">
+        <is>
+          <t>Metro</t>
+        </is>
+      </c>
+      <c r="B15" s="71" t="inlineStr">
+        <is>
+          <t>7 Days Inn Maluwan</t>
+        </is>
+      </c>
+      <c r="C15" s="78" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="D15" s="71" t="n">
+        <v>45</v>
+      </c>
+      <c r="E15" s="71" t="inlineStr">
+        <is>
+          <t>Qingnian Dajie (L1/L2) (0.62)</t>
+        </is>
+      </c>
+      <c r="F15" s="71" t="inlineStr">
+        <is>
+          <t>35 (L2&gt;L3, 3 stops, 1 change)</t>
+        </is>
+      </c>
+      <c r="G15" s="71" t="inlineStr">
+        <is>
+          <t>13 / ¥10</t>
+        </is>
+      </c>
+      <c r="H15" s="79" t="n">
+        <v>87</v>
+      </c>
+      <c r="I15" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J15" s="80">
+        <f>H15*IF(I15="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K15" s="71" t="inlineStr">
+        <is>
+          <t>no reviews</t>
+        </is>
+      </c>
+      <c r="L15" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Trip.com, 22 Oct. chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="71" t="inlineStr">
+        <is>
+          <t>Metro</t>
+        </is>
+      </c>
+      <c r="B16" s="71" t="inlineStr">
+        <is>
+          <t>Hanting Express Bus Station North</t>
+        </is>
+      </c>
+      <c r="C16" s="78" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="D16" s="71" t="n">
+        <v>46</v>
+      </c>
+      <c r="E16" s="71" t="inlineStr">
+        <is>
+          <t>Nanta (L3) (0.40)</t>
+        </is>
+      </c>
+      <c r="F16" s="71" t="inlineStr">
+        <is>
+          <t>26 (L3, 3 stops)</t>
+        </is>
+      </c>
+      <c r="G16" s="71" t="inlineStr">
+        <is>
+          <t>13 / ¥10</t>
+        </is>
+      </c>
+      <c r="H16" s="79" t="n">
+        <v>95</v>
+      </c>
+      <c r="I16" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J16" s="80">
+        <f>H16*IF(I16="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K16" s="71" t="inlineStr">
+        <is>
+          <t>TA 3.0 (1)</t>
+        </is>
+      </c>
+      <c r="L16" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Trip.com (1 room, 3 ppl), 22 Oct. chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="71" t="inlineStr">
+        <is>
+          <t>Metro</t>
+        </is>
+      </c>
+      <c r="B17" s="71" t="inlineStr">
+        <is>
+          <t>Jianing Apartment Hotel Wenhua Rd</t>
+        </is>
+      </c>
+      <c r="C17" s="78" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D17" s="71" t="n">
+        <v>52</v>
+      </c>
+      <c r="E17" s="71" t="inlineStr">
+        <is>
+          <t>Qingnian Dajie (L1/L2) (0.35)</t>
+        </is>
+      </c>
+      <c r="F17" s="71" t="inlineStr">
+        <is>
+          <t>30 (L2&gt;L3, 3 stops, 1 change)</t>
+        </is>
+      </c>
+      <c r="G17" s="71" t="inlineStr">
+        <is>
+          <t>14 / ¥11</t>
+        </is>
+      </c>
+      <c r="H17" s="79" t="n">
+        <v>103</v>
+      </c>
+      <c r="I17" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J17" s="80">
+        <f>H17*IF(I17="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K17" s="71" t="inlineStr">
+        <is>
+          <t>no reviews</t>
+        </is>
+      </c>
+      <c r="L17" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Trip.com, 22 Oct. apartment</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="71" t="inlineStr">
+        <is>
+          <t>Metro</t>
+        </is>
+      </c>
+      <c r="B18" s="71" t="inlineStr">
+        <is>
+          <t>Moon Hotel</t>
+        </is>
+      </c>
+      <c r="C18" s="78" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="D18" s="71" t="n">
+        <v>42</v>
+      </c>
+      <c r="E18" s="71" t="inlineStr">
+        <is>
+          <t>Qingnian Gongyuan (L2) (0.44)</t>
+        </is>
+      </c>
+      <c r="F18" s="71" t="inlineStr">
+        <is>
+          <t>30 (L2&gt;L3, 2 stops, 1 change)</t>
+        </is>
+      </c>
+      <c r="G18" s="71" t="inlineStr">
+        <is>
+          <t>12 / ¥10</t>
+        </is>
+      </c>
+      <c r="H18" s="79" t="n">
+        <v>106</v>
+      </c>
+      <c r="I18" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J18" s="80">
+        <f>H18*IF(I18="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K18" s="71" t="inlineStr">
+        <is>
+          <t>no reviews</t>
+        </is>
+      </c>
+      <c r="L18" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Trip.com, 22 Oct. independent</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="71" t="inlineStr">
+        <is>
+          <t>Metro</t>
+        </is>
+      </c>
+      <c r="B19" s="71" t="inlineStr">
+        <is>
+          <t>LazyBee International Youth Hostel</t>
+        </is>
+      </c>
+      <c r="C19" s="78" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="D19" s="71" t="n">
+        <v>47</v>
+      </c>
+      <c r="E19" s="71" t="inlineStr">
+        <is>
+          <t>Qingnian Dajie (L1/L2) (0.12)</t>
+        </is>
+      </c>
+      <c r="F19" s="71" t="inlineStr">
+        <is>
+          <t>27 (L2&gt;L3, 3 stops, 1 change)</t>
+        </is>
+      </c>
+      <c r="G19" s="71" t="inlineStr">
+        <is>
+          <t>13 / ¥11</t>
+        </is>
+      </c>
+      <c r="H19" s="79" t="n">
+        <v>112</v>
+      </c>
+      <c r="I19" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J19" s="80">
+        <f>H19*IF(I19="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K19" s="71" t="inlineStr">
+        <is>
+          <t>TA 4.3 (8)</t>
+        </is>
+      </c>
+      <c r="L19" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Trip.com, 22 Oct. hostel, private rooms</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="71" t="inlineStr">
+        <is>
+          <t>Metro</t>
+        </is>
+      </c>
+      <c r="B20" s="71" t="inlineStr">
+        <is>
+          <t>Home Inn Neo Railway Stn Nanwu Rd Metro</t>
+        </is>
+      </c>
+      <c r="C20" s="78" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="D20" s="71" t="n">
+        <v>39</v>
+      </c>
+      <c r="E20" s="71" t="inlineStr">
+        <is>
+          <t>Jiaxing Jie (L3) (0.81)</t>
+        </is>
+      </c>
+      <c r="F20" s="71" t="inlineStr">
+        <is>
+          <t>31 (L3, 2 stops)</t>
+        </is>
+      </c>
+      <c r="G20" s="71" t="inlineStr">
+        <is>
+          <t>12 / ¥9</t>
+        </is>
+      </c>
+      <c r="H20" s="79" t="n">
+        <v>117</v>
+      </c>
+      <c r="I20" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J20" s="80">
+        <f>H20*IF(I20="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K20" s="71" t="inlineStr">
+        <is>
+          <t>TA 3.8 (93)</t>
+        </is>
+      </c>
+      <c r="L20" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Agoda, 22 Oct. chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="71" t="inlineStr">
+        <is>
+          <t>Metro</t>
+        </is>
+      </c>
+      <c r="B21" s="71" t="inlineStr">
+        <is>
+          <t>Home Inn Nanta</t>
+        </is>
+      </c>
+      <c r="C21" s="78" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="D21" s="71" t="n">
+        <v>55</v>
+      </c>
+      <c r="E21" s="71" t="inlineStr">
+        <is>
+          <t>Wenfu Lu (L3) (0.45)</t>
+        </is>
+      </c>
+      <c r="F21" s="71" t="inlineStr">
+        <is>
+          <t>29 (L3, 4 stops)</t>
+        </is>
+      </c>
+      <c r="G21" s="71" t="inlineStr">
+        <is>
+          <t>15 / ¥12</t>
+        </is>
+      </c>
+      <c r="H21" s="79" t="n">
+        <v>139</v>
+      </c>
+      <c r="I21" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J21" s="80">
+        <f>H21*IF(I21="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K21" s="71" t="inlineStr">
+        <is>
+          <t>TA 3.9 (134)</t>
+        </is>
+      </c>
+      <c r="L21" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Trip.com, 22 Oct. chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="76" t="inlineStr">
+        <is>
+          <t>TAXI – no handy metro (or two changes); 13–30 min, ¥10–23 per car</t>
+        </is>
+      </c>
+      <c r="B22" s="77" t="n"/>
+      <c r="C22" s="77" t="n"/>
+      <c r="D22" s="77" t="n"/>
+      <c r="E22" s="77" t="n"/>
+      <c r="F22" s="77" t="n"/>
+      <c r="G22" s="77" t="n"/>
+      <c r="H22" s="77" t="n"/>
+      <c r="I22" s="77" t="n"/>
+      <c r="J22" s="77" t="n"/>
+      <c r="K22" s="77" t="n"/>
+      <c r="L22" s="77" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="71" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="B23" s="71" t="inlineStr">
+        <is>
+          <t>YDOO &amp; YGOO Hotel</t>
+        </is>
+      </c>
+      <c r="C23" s="78" t="n">
+        <v>5.38</v>
+      </c>
+      <c r="D23" s="71" t="n">
+        <v>90</v>
+      </c>
+      <c r="E23" s="71" t="inlineStr">
+        <is>
+          <t>Jinrong Zhongxin (L2) (0.90)</t>
+        </is>
+      </c>
+      <c r="F23" s="71" t="inlineStr">
+        <is>
+          <t>44 (L2&gt;L3, 5 stops, 1 change)</t>
+        </is>
+      </c>
+      <c r="G23" s="71" t="inlineStr">
+        <is>
+          <t>23 / ¥18</t>
+        </is>
+      </c>
+      <c r="H23" s="79" t="n">
+        <v>58</v>
+      </c>
+      <c r="I23" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J23" s="80">
+        <f>H23*IF(I23="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K23" s="71" t="inlineStr">
+        <is>
+          <t>no reviews</t>
+        </is>
+      </c>
+      <c r="L23" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Vio, 22 Oct. independent</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="71" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="B24" s="71" t="inlineStr">
+        <is>
+          <t>Shenyang Dongdong Hotel</t>
+        </is>
+      </c>
+      <c r="C24" s="78" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="D24" s="71" t="n">
+        <v>121</v>
+      </c>
+      <c r="E24" s="71" t="inlineStr">
+        <is>
+          <t>none within 1 km</t>
+        </is>
+      </c>
+      <c r="F24" s="71" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G24" s="71" t="inlineStr">
+        <is>
+          <t>30 / ¥23</t>
+        </is>
+      </c>
+      <c r="H24" s="79" t="n">
+        <v>58</v>
+      </c>
+      <c r="I24" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J24" s="80">
+        <f>H24*IF(I24="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K24" s="71" t="inlineStr">
+        <is>
+          <t>no reviews</t>
+        </is>
+      </c>
+      <c r="L24" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Trip.com, 22 Oct. independent</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="71" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="B25" s="71" t="inlineStr">
+        <is>
+          <t>Xinting Hotel</t>
+        </is>
+      </c>
+      <c r="C25" s="78" t="n">
+        <v>5.39</v>
+      </c>
+      <c r="D25" s="71" t="n">
+        <v>90</v>
+      </c>
+      <c r="E25" s="71" t="inlineStr">
+        <is>
+          <t>none within 1 km</t>
+        </is>
+      </c>
+      <c r="F25" s="71" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G25" s="71" t="inlineStr">
+        <is>
+          <t>23 / ¥18</t>
+        </is>
+      </c>
+      <c r="H25" s="79" t="n">
+        <v>60</v>
+      </c>
+      <c r="I25" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J25" s="80">
+        <f>H25*IF(I25="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K25" s="71" t="inlineStr">
+        <is>
+          <t>no reviews</t>
+        </is>
+      </c>
+      <c r="L25" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Trip.com, 22 Oct. independent</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="71" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="B26" s="71" t="inlineStr">
+        <is>
+          <t>Home Inn North Station South Exit</t>
+        </is>
+      </c>
+      <c r="C26" s="78" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="D26" s="71" t="n">
+        <v>119</v>
+      </c>
+      <c r="E26" s="71" t="inlineStr">
+        <is>
+          <t>none within 1 km</t>
+        </is>
+      </c>
+      <c r="F26" s="71" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G26" s="71" t="inlineStr">
+        <is>
+          <t>29 / ¥22</t>
+        </is>
+      </c>
+      <c r="H26" s="79" t="n">
+        <v>69</v>
+      </c>
+      <c r="I26" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J26" s="80">
+        <f>H26*IF(I26="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K26" s="71" t="inlineStr">
+        <is>
+          <t>no reviews</t>
+        </is>
+      </c>
+      <c r="L26" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Vio, 22 Oct. chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="71" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="B27" s="71" t="inlineStr">
+        <is>
+          <t>Jinjiang Inn Shenyang North Station</t>
+        </is>
+      </c>
+      <c r="C27" s="78" t="n">
+        <v>6.88</v>
+      </c>
+      <c r="D27" s="71" t="n">
+        <v>115</v>
+      </c>
+      <c r="E27" s="71" t="inlineStr">
+        <is>
+          <t>none within 1 km</t>
+        </is>
+      </c>
+      <c r="F27" s="71" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G27" s="71" t="inlineStr">
+        <is>
+          <t>28 / ¥22</t>
+        </is>
+      </c>
+      <c r="H27" s="79" t="n">
+        <v>71</v>
+      </c>
+      <c r="I27" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J27" s="80">
+        <f>H27*IF(I27="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K27" s="71" t="inlineStr">
+        <is>
+          <t>TA 4.3 (84)</t>
+        </is>
+      </c>
+      <c r="L27" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Trip.com, 22 Oct. chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="71" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="B28" s="71" t="inlineStr">
+        <is>
+          <t>Bestay Express Huaiyuanmen</t>
+        </is>
+      </c>
+      <c r="C28" s="78" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D28" s="71" t="n">
+        <v>70</v>
+      </c>
+      <c r="E28" s="71" t="inlineStr">
+        <is>
+          <t>Huaiyuanmen (L1) (0.45)</t>
+        </is>
+      </c>
+      <c r="F28" s="71" t="inlineStr">
+        <is>
+          <t>39 (L1&gt;L2&gt;L3, 4 stops, 2 changes)</t>
+        </is>
+      </c>
+      <c r="G28" s="71" t="inlineStr">
+        <is>
+          <t>18 / ¥14</t>
+        </is>
+      </c>
+      <c r="H28" s="79" t="n">
+        <v>77</v>
+      </c>
+      <c r="I28" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J28" s="80">
+        <f>H28*IF(I28="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K28" s="71" t="inlineStr">
+        <is>
+          <t>Booking 7.5 (7); TA 4.7 (3)</t>
+        </is>
+      </c>
+      <c r="L28" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Booking.com, 22 Oct. Booking.com direct ¥516 (2 rooms) / ¥266 (1 room for 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="71" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="B29" s="71" t="inlineStr">
+        <is>
+          <t>Jinshang Express Motel</t>
+        </is>
+      </c>
+      <c r="C29" s="78" t="n">
+        <v>4.28</v>
+      </c>
+      <c r="D29" s="71" t="n">
+        <v>71</v>
+      </c>
+      <c r="E29" s="71" t="inlineStr">
+        <is>
+          <t>Shenyang Stn (L1) (0.94)</t>
+        </is>
+      </c>
+      <c r="F29" s="71" t="inlineStr">
+        <is>
+          <t>52 (L1&gt;L2&gt;L3, 6 stops, 2 changes)</t>
+        </is>
+      </c>
+      <c r="G29" s="71" t="inlineStr">
+        <is>
+          <t>19 / ¥15</t>
+        </is>
+      </c>
+      <c r="H29" s="79" t="n">
+        <v>81</v>
+      </c>
+      <c r="I29" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J29" s="80">
+        <f>H29*IF(I29="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K29" s="71" t="inlineStr">
+        <is>
+          <t>no reviews</t>
+        </is>
+      </c>
+      <c r="L29" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Trip.com, 22 Oct. independent</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="71" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="B30" s="71" t="inlineStr">
+        <is>
+          <t>7 Days Premium Railway Stn Zhongshan Sq</t>
+        </is>
+      </c>
+      <c r="C30" s="78" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="D30" s="71" t="n">
+        <v>61</v>
+      </c>
+      <c r="E30" s="71" t="inlineStr">
+        <is>
+          <t>none within 1 km</t>
+        </is>
+      </c>
+      <c r="F30" s="71" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G30" s="71" t="inlineStr">
+        <is>
+          <t>16 / ¥13</t>
+        </is>
+      </c>
+      <c r="H30" s="79" t="n">
+        <v>86</v>
+      </c>
+      <c r="I30" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J30" s="80">
+        <f>H30*IF(I30="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K30" s="71" t="inlineStr">
+        <is>
+          <t>TA 4.1 (83)</t>
+        </is>
+      </c>
+      <c r="L30" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Trip.com, 22 Oct. chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="71" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="B31" s="71" t="inlineStr">
+        <is>
+          <t>7 Days Inn Gugong Huaiyuanmen</t>
+        </is>
+      </c>
+      <c r="C31" s="78" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="D31" s="71" t="n">
+        <v>69</v>
+      </c>
+      <c r="E31" s="71" t="inlineStr">
+        <is>
+          <t>Huaiyuanmen (L1) (0.44)</t>
+        </is>
+      </c>
+      <c r="F31" s="71" t="inlineStr">
+        <is>
+          <t>39 (L1&gt;L2&gt;L3, 4 stops, 2 changes)</t>
+        </is>
+      </c>
+      <c r="G31" s="71" t="inlineStr">
+        <is>
+          <t>18 / ¥14</t>
+        </is>
+      </c>
+      <c r="H31" s="79" t="n">
+        <v>91</v>
+      </c>
+      <c r="I31" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J31" s="80">
+        <f>H31*IF(I31="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K31" s="71" t="inlineStr">
+        <is>
+          <t>TA 4.3 (7)</t>
+        </is>
+      </c>
+      <c r="L31" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Trip.com, 22 Oct. chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="71" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="B32" s="71" t="inlineStr">
+        <is>
+          <t>GreenTree Inn Tiexi Yunfeng St</t>
+        </is>
+      </c>
+      <c r="C32" s="78" t="n">
+        <v>4.51</v>
+      </c>
+      <c r="D32" s="71" t="n">
+        <v>75</v>
+      </c>
+      <c r="E32" s="71" t="inlineStr">
+        <is>
+          <t>Yunfeng Beijie (L1) (0.32)</t>
+        </is>
+      </c>
+      <c r="F32" s="71" t="inlineStr">
+        <is>
+          <t>44 (L1&gt;L2&gt;L3, 7 stops, 2 changes)</t>
+        </is>
+      </c>
+      <c r="G32" s="71" t="inlineStr">
+        <is>
+          <t>20 / ¥15</t>
+        </is>
+      </c>
+      <c r="H32" s="79" t="n">
+        <v>91</v>
+      </c>
+      <c r="I32" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J32" s="80">
+        <f>H32*IF(I32="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K32" s="71" t="inlineStr">
+        <is>
+          <t>no reviews</t>
+        </is>
+      </c>
+      <c r="L32" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Vio, 22 Oct. chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="71" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="B33" s="71" t="inlineStr">
+        <is>
+          <t>Jinjiang Inn Select Taiyuan South St</t>
+        </is>
+      </c>
+      <c r="C33" s="78" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="D33" s="71" t="n">
+        <v>43</v>
+      </c>
+      <c r="E33" s="71" t="inlineStr">
+        <is>
+          <t>Taiyuan Jie (L1) (0.76)</t>
+        </is>
+      </c>
+      <c r="F33" s="71" t="inlineStr">
+        <is>
+          <t>47 (L1&gt;L2&gt;L3, 5 stops, 2 changes)</t>
+        </is>
+      </c>
+      <c r="G33" s="71" t="inlineStr">
+        <is>
+          <t>13 / ¥10</t>
+        </is>
+      </c>
+      <c r="H33" s="79" t="n">
+        <v>99</v>
+      </c>
+      <c r="I33" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J33" s="80">
+        <f>H33*IF(I33="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K33" s="71" t="inlineStr">
+        <is>
+          <t>no reviews</t>
+        </is>
+      </c>
+      <c r="L33" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Priceline, 22 Oct. chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="71" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="B34" s="71" t="inlineStr">
+        <is>
+          <t>Jinjiang Inn North Rly Stn Huigong Sq (Booking)</t>
+        </is>
+      </c>
+      <c r="C34" s="78" t="n">
+        <v>6.36</v>
+      </c>
+      <c r="D34" s="71" t="n">
+        <v>106</v>
+      </c>
+      <c r="E34" s="71" t="inlineStr">
+        <is>
+          <t>none within 1 km</t>
+        </is>
+      </c>
+      <c r="F34" s="71" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G34" s="71" t="inlineStr">
+        <is>
+          <t>26 / ¥20</t>
+        </is>
+      </c>
+      <c r="H34" s="79" t="n">
+        <v>804</v>
+      </c>
+      <c r="I34" s="71" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J34" s="80">
+        <f>H34*IF(I34="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K34" s="71" t="inlineStr">
+        <is>
+          <t>Booking 7.0 (5)</t>
+        </is>
+      </c>
+      <c r="L34" s="71" t="inlineStr">
+        <is>
+          <t>Booking.com, 22 Oct. chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="71" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="B35" s="71" t="inlineStr">
+        <is>
+          <t>7Days Premium Olympic Sports Center</t>
+        </is>
+      </c>
+      <c r="C35" s="78" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="D35" s="71" t="n">
+        <v>65</v>
+      </c>
+      <c r="E35" s="71" t="inlineStr">
+        <is>
+          <t>none within 1 km</t>
+        </is>
+      </c>
+      <c r="F35" s="71" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G35" s="71" t="inlineStr">
+        <is>
+          <t>17 / ¥13</t>
+        </is>
+      </c>
+      <c r="H35" s="79" t="n">
+        <v>128</v>
+      </c>
+      <c r="I35" s="71" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J35" s="80">
+        <f>H35*IF(I35="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K35" s="71" t="inlineStr">
+        <is>
+          <t>Booking 8.5 (2)</t>
+        </is>
+      </c>
+      <c r="L35" s="71" t="inlineStr">
+        <is>
+          <t>Tripadvisor→Booking.com, 22 Oct. Booking.com direct ¥906 (2 rooms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="71" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="B36" s="71" t="inlineStr">
+        <is>
+          <t>Jinjiang Inn Zhongshan Sq / Med Univ 1st Hosp (Booking)</t>
+        </is>
+      </c>
+      <c r="C36" s="78" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="D36" s="71" t="n">
+        <v>61</v>
+      </c>
+      <c r="E36" s="71" t="inlineStr">
+        <is>
+          <t>Renmin Guangchang (L2) (0.99)</t>
+        </is>
+      </c>
+      <c r="F36" s="71" t="inlineStr">
+        <is>
+          <t>43 (L2&gt;L3, 4 stops, 1 change)</t>
+        </is>
+      </c>
+      <c r="G36" s="71" t="inlineStr">
+        <is>
+          <t>16 / ¥13</t>
+        </is>
+      </c>
+      <c r="H36" s="79" t="n">
+        <v>924</v>
+      </c>
+      <c r="I36" s="71" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J36" s="80">
+        <f>H36*IF(I36="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K36" s="71" t="inlineStr">
+        <is>
+          <t>Booking 8.3 (3)</t>
+        </is>
+      </c>
+      <c r="L36" s="71" t="inlineStr">
+        <is>
+          <t>Booking.com (1 room, 3 ppl), 22 Oct. chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="76" t="inlineStr">
+        <is>
+          <t>EARLIER TRIP.COM CHECKS NEAR NEU (from the built-in browser; prices as seen then)</t>
+        </is>
+      </c>
+      <c r="B37" s="77" t="n"/>
+      <c r="C37" s="77" t="n"/>
+      <c r="D37" s="77" t="n"/>
+      <c r="E37" s="77" t="n"/>
+      <c r="F37" s="77" t="n"/>
+      <c r="G37" s="77" t="n"/>
+      <c r="H37" s="77" t="n"/>
+      <c r="I37" s="77" t="n"/>
+      <c r="J37" s="77" t="n"/>
+      <c r="K37" s="77" t="n"/>
+      <c r="L37" s="77" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="71" t="inlineStr">
+        <is>
+          <t>Walk</t>
+        </is>
+      </c>
+      <c r="B38" s="71" t="inlineStr">
+        <is>
+          <t>Aiyi Future Serviced Apartment – Family 2-bed room for 4</t>
+        </is>
+      </c>
+      <c r="C38" s="71" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D38" s="71" t="n"/>
+      <c r="E38" s="71" t="n"/>
+      <c r="F38" s="71" t="n"/>
+      <c r="G38" s="71" t="n"/>
+      <c r="H38" s="79" t="n">
+        <v>528</v>
+      </c>
+      <c r="I38" s="71" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J38" s="80">
+        <f>H38*IF(I38="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K38" s="71" t="inlineStr">
+        <is>
+          <t>9.8 (957)</t>
+        </is>
+      </c>
+      <c r="L38" s="71" t="inlineStr">
+        <is>
+          <t>Trip.com 1 Oct, 12–15 Nov, 1 room for 4. Cheapest well-rated option; re-check before booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="71" t="inlineStr">
+        <is>
+          <t>Walk</t>
+        </is>
+      </c>
+      <c r="B39" s="71" t="inlineStr">
+        <is>
+          <t>Shenyang RiCH Hotel (Sanhao St) – Family Room</t>
+        </is>
+      </c>
+      <c r="C39" s="71" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D39" s="71" t="n"/>
+      <c r="E39" s="71" t="n"/>
+      <c r="F39" s="71" t="n"/>
+      <c r="G39" s="71" t="n"/>
+      <c r="H39" s="79" t="n">
+        <v>976</v>
+      </c>
+      <c r="I39" s="71" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J39" s="80">
+        <f>H39*IF(I39="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K39" s="71" t="inlineStr">
+        <is>
+          <t>9.6 (1,802)</t>
+        </is>
+      </c>
+      <c r="L39" s="71" t="inlineStr">
+        <is>
+          <t>Trip.com 1 Oct, 1 room for 3 or 4 (used in Shenyang – Comfort)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="71" t="inlineStr">
+        <is>
+          <t>Walk</t>
+        </is>
+      </c>
+      <c r="B40" s="71" t="inlineStr">
+        <is>
+          <t>Jinke Hotel – 2 rooms (double beds)</t>
+        </is>
+      </c>
+      <c r="C40" s="71" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="D40" s="71" t="n"/>
+      <c r="E40" s="71" t="n"/>
+      <c r="F40" s="71" t="n"/>
+      <c r="G40" s="71" t="n"/>
+      <c r="H40" s="79" t="n">
+        <v>1044</v>
+      </c>
+      <c r="I40" s="71" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J40" s="80">
+        <f>H40*IF(I40="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K40" s="71" t="inlineStr">
+        <is>
+          <t>9.6</t>
+        </is>
+      </c>
+      <c r="L40" s="71" t="inlineStr">
+        <is>
+          <t>Trip.com 22 Oct; same hotel as Jin Ke above</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="71" t="inlineStr">
+        <is>
+          <t>Walk</t>
+        </is>
+      </c>
+      <c r="B41" s="71" t="inlineStr">
+        <is>
+          <t>Birches Hotel – 2 rooms (double beds, windowless)</t>
+        </is>
+      </c>
+      <c r="C41" s="71" t="n"/>
+      <c r="D41" s="71" t="n"/>
+      <c r="E41" s="71" t="n"/>
+      <c r="F41" s="71" t="n"/>
+      <c r="G41" s="71" t="n"/>
+      <c r="H41" s="79" t="n">
+        <v>1116</v>
+      </c>
+      <c r="I41" s="71" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J41" s="80">
+        <f>H41*IF(I41="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K41" s="71" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="L41" s="71" t="inlineStr">
+        <is>
+          <t>Trip.com 22 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="71" t="inlineStr">
+        <is>
+          <t>Walk</t>
+        </is>
+      </c>
+      <c r="B42" s="71" t="inlineStr">
+        <is>
+          <t>RiCH Hotel – 2 Forest Rooms</t>
+        </is>
+      </c>
+      <c r="C42" s="71" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D42" s="71" t="n"/>
+      <c r="E42" s="71" t="n"/>
+      <c r="F42" s="71" t="n"/>
+      <c r="G42" s="71" t="n"/>
+      <c r="H42" s="79" t="n">
+        <v>1220</v>
+      </c>
+      <c r="I42" s="71" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J42" s="80">
+        <f>H42*IF(I42="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K42" s="71" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="L42" s="71" t="inlineStr">
+        <is>
+          <t>Trip.com 22 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="71" t="inlineStr">
+        <is>
+          <t>Walk</t>
+        </is>
+      </c>
+      <c r="B43" s="71" t="inlineStr">
+        <is>
+          <t>Ji Hotel Sanhao St – 2 Budget Twin rooms</t>
+        </is>
+      </c>
+      <c r="C43" s="71" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="D43" s="71" t="n"/>
+      <c r="E43" s="71" t="n"/>
+      <c r="F43" s="71" t="n"/>
+      <c r="G43" s="71" t="n"/>
+      <c r="H43" s="79" t="n">
+        <v>1371</v>
+      </c>
+      <c r="I43" s="71" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J43" s="80">
+        <f>H43*IF(I43="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K43" s="71" t="inlineStr">
+        <is>
+          <t>9.0 (1,433)</t>
+        </is>
+      </c>
+      <c r="L43" s="71" t="inlineStr">
+        <is>
+          <t>Trip.com 22 Oct; twin beds (used in Shenyang – Sleep value)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="71" t="inlineStr">
+        <is>
+          <t>Walk</t>
+        </is>
+      </c>
+      <c r="B44" s="71" t="inlineStr">
+        <is>
+          <t>Lavande Hotel – 2 rooms</t>
+        </is>
+      </c>
+      <c r="C44" s="71" t="n"/>
+      <c r="D44" s="71" t="n"/>
+      <c r="E44" s="71" t="n"/>
+      <c r="F44" s="71" t="n"/>
+      <c r="G44" s="71" t="n"/>
+      <c r="H44" s="79" t="n">
+        <v>1410</v>
+      </c>
+      <c r="I44" s="71" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J44" s="80">
+        <f>H44*IF(I44="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K44" s="71" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="L44" s="71" t="inlineStr">
+        <is>
+          <t>Trip.com 22 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="71" t="inlineStr">
+        <is>
+          <t>Walk</t>
+        </is>
+      </c>
+      <c r="B45" s="71" t="inlineStr">
+        <is>
+          <t>NEU International (on campus) – 2 Superior Twin</t>
+        </is>
+      </c>
+      <c r="C45" s="71" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="D45" s="71" t="n"/>
+      <c r="E45" s="71" t="n"/>
+      <c r="F45" s="71" t="n"/>
+      <c r="G45" s="71" t="n"/>
+      <c r="H45" s="79" t="n">
+        <v>2388</v>
+      </c>
+      <c r="I45" s="71" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J45" s="80">
+        <f>H45*IF(I45="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K45" s="71" t="inlineStr">
+        <is>
+          <t>9.7 (1,998)</t>
+        </is>
+      </c>
+      <c r="L45" s="71" t="inlineStr">
+        <is>
+          <t>Trip.com 22 Oct, 30% 'Surprise Savings' rate (used in Shenyang – Sleep first)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="71" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="B46" s="71" t="inlineStr">
+        <is>
+          <t>Bestay Hotel Express Huaiyuanmen – 2 Family Rooms (2 nights)</t>
+        </is>
+      </c>
+      <c r="C46" s="71" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D46" s="71" t="n"/>
+      <c r="E46" s="71" t="n"/>
+      <c r="F46" s="71" t="n"/>
+      <c r="G46" s="71" t="n"/>
+      <c r="H46" s="79" t="n">
+        <v>284</v>
+      </c>
+      <c r="I46" s="71" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J46" s="80">
+        <f>H46*IF(I46="USD",$B$3,$D$3)</f>
+        <v/>
+      </c>
+      <c r="K46" s="71" t="inlineStr">
+        <is>
+          <t>8.2 (1,062)</t>
+        </is>
+      </c>
+      <c r="L46" s="71" t="inlineStr">
+        <is>
+          <t>Trip.com 1 Oct, 13–15 Nov; Booking.com 22 Oct ¥516 for 3 nights</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="72" t="inlineStr">
+        <is>
+          <t>Commute cost check</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1" s="26">
+      <c r="A49" s="71" t="inlineStr">
+        <is>
+          <t>Trips to campus: 14 Nov there and back, 15 Nov there and back (luggage stays at the hotel after the contest-morning check-out) = 4 trips.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1" s="26">
+      <c r="A50" s="71" t="inlineStr">
+        <is>
+          <t>Taxi for the whole team (one car for 3–4 people): 4 × ¥9–23 = ¥36–92 (₮19–49k). Metro: ¥2–4 per person per ride, 4 people × 4 rides = ¥32–64, so with 3–4 people a taxi costs about the same as the metro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1" s="26">
+      <c r="A51" s="71" t="inlineStr">
+        <is>
+          <t>Cheapest walkable chain (7 Days Inn Sanhao St Liaozhan $95 ≈ ₮342k) vs cheapest taxi-distance chains (Jinjiang Inn North Station $71 ≈ ₮255k, Bestay Huaiyuanmen ¥516 ≈ ₮277k) + 4 taxi rides (¥56–88): only ~₮35–40k saved for the whole team (₮10–13k per person), ~₮95k with the no-review $58 hotels, for a 20–30 min commute on contest morning. The sleep rule favours the walk group.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1" s="26">
+      <c r="A52" s="81" t="inlineStr">
+        <is>
+          <t>ASSUMPTION: taxi tariff ¥9 for 3 km + ¥2/km and the metro time model above. Didi (app or Alipay mini-program) is usually the same price or cheaper than a street taxi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="72" t="inlineStr">
+        <is>
+          <t>Metro stations near NEU (OpenStreetMap / Nominatim, 22 Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="82" t="inlineStr">
+        <is>
+          <t>Station</t>
+        </is>
+      </c>
+      <c r="B55" s="82" t="inlineStr">
+        <is>
+          <t>Lines</t>
+        </is>
+      </c>
+      <c r="C55" s="82" t="inlineStr">
+        <is>
+          <t>Lat</t>
+        </is>
+      </c>
+      <c r="D55" s="82" t="inlineStr">
+        <is>
+          <t>Lon</t>
+        </is>
+      </c>
+      <c r="E55" s="82" t="inlineStr">
+        <is>
+          <t>Distance to NEU (km)</t>
+        </is>
+      </c>
+      <c r="F55" s="82" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="74" t="inlineStr">
+        <is>
+          <t>Sanhaojie 三好街</t>
+        </is>
+      </c>
+      <c r="B56" s="74" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="C56" s="74" t="n">
+        <v>41.7691</v>
+      </c>
+      <c r="D56" s="74" t="n">
+        <v>123.4222</v>
+      </c>
+      <c r="E56" s="74" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F56" s="74" t="inlineStr">
+        <is>
+          <t>Nearest to NEU; Wenhua Road</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="74" t="inlineStr">
+        <is>
+          <t>Fangxing Guangchang 方型广场</t>
+        </is>
+      </c>
+      <c r="B57" s="74" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="C57" s="74" t="n">
+        <v>41.7723</v>
+      </c>
+      <c r="D57" s="74" t="n">
+        <v>123.4101</v>
+      </c>
+      <c r="E57" s="74" t="n">
+        <v>1</v>
+      </c>
+      <c r="F57" s="74" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="74" t="inlineStr">
+        <is>
+          <t>Gongye Zhanlanguan 工业展览馆</t>
+        </is>
+      </c>
+      <c r="B58" s="74" t="inlineStr">
+        <is>
+          <t>L2 / L3</t>
+        </is>
+      </c>
+      <c r="C58" s="74" t="n">
+        <v>41.7709</v>
+      </c>
+      <c r="D58" s="74" t="n">
+        <v>123.4293</v>
+      </c>
+      <c r="E58" s="74" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F58" s="74" t="inlineStr">
+        <is>
+          <t>Change L2 ⇄ L3 (or walk ~1 km to campus)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="74" t="inlineStr">
+        <is>
+          <t>Shi Tushuguan 市图书馆</t>
+        </is>
+      </c>
+      <c r="B59" s="74" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C59" s="74" t="n">
+        <v>41.7576</v>
+      </c>
+      <c r="D59" s="74" t="n">
+        <v>123.4293</v>
+      </c>
+      <c r="E59" s="74" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F59" s="74" t="inlineStr">
+        <is>
+          <t>Approach from the south-east</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="74" t="inlineStr">
+        <is>
+          <t>Jiaxing Jie 嘉兴街</t>
+        </is>
+      </c>
+      <c r="B60" s="74" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="C60" s="74" t="n">
+        <v>41.7747</v>
+      </c>
+      <c r="D60" s="74" t="n">
+        <v>123.4046</v>
+      </c>
+      <c r="E60" s="74" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F60" s="74" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="74" t="inlineStr">
+        <is>
+          <t>Zhongkeyuan Jinshusuo 中科院金属所</t>
+        </is>
+      </c>
+      <c r="B61" s="74" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="C61" s="74" t="n">
+        <v>41.7687</v>
+      </c>
+      <c r="D61" s="74" t="n">
+        <v>123.438</v>
+      </c>
+      <c r="E61" s="74" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="F61" s="74" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="74" t="inlineStr">
+        <is>
+          <t>Qingnian Gongyuan 青年公园</t>
+        </is>
+      </c>
+      <c r="B62" s="74" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C62" s="74" t="n">
+        <v>41.7824</v>
+      </c>
+      <c r="D62" s="74" t="n">
+        <v>123.4297</v>
+      </c>
+      <c r="E62" s="74" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F62" s="74" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="74" t="inlineStr">
+        <is>
+          <t>Nanta 南塔</t>
+        </is>
+      </c>
+      <c r="B63" s="74" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="C63" s="74" t="n">
+        <v>41.7685</v>
+      </c>
+      <c r="D63" s="74" t="n">
+        <v>123.4467</v>
+      </c>
+      <c r="E63" s="74" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F63" s="74" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="74" t="inlineStr">
+        <is>
+          <t>Nanshichang 南市场</t>
+        </is>
+      </c>
+      <c r="B64" s="74" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C64" s="74" t="n">
+        <v>41.787</v>
+      </c>
+      <c r="D64" s="74" t="n">
+        <v>123.4138</v>
+      </c>
+      <c r="E64" s="74" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F64" s="74" t="inlineStr">
+        <is>
+          <t>L1 → L2 at Qingnian Dajie → L3</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="74" t="inlineStr">
+        <is>
+          <t>Shayang 砂阳</t>
+        </is>
+      </c>
+      <c r="B65" s="74" t="inlineStr">
+        <is>
+          <t>L3 / L4</t>
+        </is>
+      </c>
+      <c r="C65" s="74" t="n">
+        <v>41.7651</v>
+      </c>
+      <c r="D65" s="74" t="n">
+        <v>123.3855</v>
+      </c>
+      <c r="E65" s="74" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="F65" s="74" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="74" t="inlineStr">
+        <is>
+          <t>Huaiyuanmen 怀远门</t>
+        </is>
+      </c>
+      <c r="B66" s="74" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C66" s="74" t="n">
+        <v>41.7946</v>
+      </c>
+      <c r="D66" s="74" t="n">
+        <v>123.4412</v>
+      </c>
+      <c r="E66" s="74" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="F66" s="74" t="inlineStr">
+        <is>
+          <t>Near Bestay / 7 Days Gugong</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="74" t="inlineStr">
+        <is>
+          <t>Shenyang North Station 沈阳北站</t>
+        </is>
+      </c>
+      <c r="B67" s="74" t="inlineStr">
+        <is>
+          <t>L2 / L4</t>
+        </is>
+      </c>
+      <c r="C67" s="74" t="n">
+        <v>41.8173</v>
+      </c>
+      <c r="D67" s="74" t="n">
+        <v>123.4297</v>
+      </c>
+      <c r="E67" s="74" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="F67" s="74" t="inlineStr">
+        <is>
+          <t>L2 to Gongye Zhanlanguan, change to L3; L2 also runs to Taoxian airport</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A52:L52"/>
+    <mergeCell ref="A51:L51"/>
+    <mergeCell ref="A49:L49"/>
+    <mergeCell ref="A50:L50"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Shenyang hotels: add Trip.com / Tripadvisor / Booking links and Trip.com checks
The "Shenyang hotels by distance" sheet gets two link columns (Trip.com
detail pages; Tripadvisor or Booking.com with 12-15 Nov, 2 rooms / 4
guests). Trip.com confirms 7 Days Inn Sanhao St (8.9/452, twin rooms,
accepts foreign guests); ratings updated for Jinke, Ji Hotel, RiCH,
Aiyi and Bestay. details.md records the Trip.com hotel ids and that
Trip.com static pages load via WebFetch from the cloud.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018GZDCacqRiEe328BLfJXxj
</commit_message>
<xml_diff>
--- a/ICPC_flight_fares_30Sep2026.xlsx
+++ b/ICPC_flight_fares_30Sep2026.xlsx
@@ -26,7 +26,7 @@
     <numFmt numFmtId="165" formatCode="#,##0&quot; ₮&quot;;\(#,##0&quot; ₮)&quot;;\-"/>
     <numFmt numFmtId="166" formatCode="#,##0&quot; ₮&quot;"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -143,6 +143,12 @@
       <color rgb="FF0000FF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF0563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -230,7 +236,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -454,6 +460,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6320,7 +6327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:N67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="26" min="1" max="1"/>
@@ -6335,6 +6342,8 @@
     <col width="13" customWidth="1" style="26" min="10" max="10"/>
     <col width="22" customWidth="1" style="26" min="11" max="11"/>
     <col width="60" customWidth="1" style="26" min="12" max="12"/>
+    <col width="11" customWidth="1" style="26" min="13" max="13"/>
+    <col width="16" customWidth="1" style="26" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6433,6 +6442,16 @@
       <c r="L5" s="75" t="inlineStr">
         <is>
           <t>Source / note</t>
+        </is>
+      </c>
+      <c r="M5" s="75" t="inlineStr">
+        <is>
+          <t>Trip.com</t>
+        </is>
+      </c>
+      <c r="N5" s="75" t="inlineStr">
+        <is>
+          <t>Tripadvisor / Booking.com (dates set)</t>
         </is>
       </c>
     </row>
@@ -6453,6 +6472,8 @@
       <c r="J6" s="77" t="n"/>
       <c r="K6" s="77" t="n"/>
       <c r="L6" s="77" t="n"/>
+      <c r="M6" s="77" t="n"/>
+      <c r="N6" s="77" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="71" t="inlineStr">
@@ -6508,6 +6529,11 @@
           <t>Tripadvisor→Booking.com, 22 Oct. chain</t>
         </is>
       </c>
+      <c r="N7" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="71" t="inlineStr">
@@ -6563,6 +6589,11 @@
           <t>Tripadvisor→Vio, 22 Oct. chain</t>
         </is>
       </c>
+      <c r="N8" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="71" t="inlineStr">
@@ -6610,12 +6641,22 @@
       </c>
       <c r="K9" s="71" t="inlineStr">
         <is>
-          <t>TA 4.0 (1)</t>
+          <t>Trip.com 8.9 (452); TA 4.0 (1)</t>
         </is>
       </c>
       <c r="L9" s="71" t="inlineStr">
         <is>
-          <t>Tripadvisor→Agoda, 22 Oct. chain</t>
+          <t>Tripadvisor→Agoda, 22 Oct. chain. Trip.com 22 Oct: 6 Jia 6 Wencui Road, Sanhaojie metro 780 m, Traditional Twin Room (2 single beds) offered, 'guests from all countries/regions are welcome'</t>
+        </is>
+      </c>
+      <c r="M9" s="83" t="inlineStr">
+        <is>
+          <t>Trip.com</t>
+        </is>
+      </c>
+      <c r="N9" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
         </is>
       </c>
     </row>
@@ -6665,12 +6706,22 @@
       </c>
       <c r="K10" s="71" t="inlineStr">
         <is>
-          <t>Trip.com 9.6; TA 3.4 (25)</t>
+          <t>Trip.com 9.5 (1,190); TA 3.4 (25)</t>
         </is>
       </c>
       <c r="L10" s="71" t="inlineStr">
         <is>
           <t>Tripadvisor→Trip.com, 22 Oct. Trip.com 22 Oct ¥1,044 for 2 rooms</t>
+        </is>
+      </c>
+      <c r="M10" s="83" t="inlineStr">
+        <is>
+          <t>Trip.com</t>
+        </is>
+      </c>
+      <c r="N10" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
         </is>
       </c>
     </row>
@@ -6726,6 +6777,11 @@
       <c r="L11" s="71" t="inlineStr">
         <is>
           <t>Booking.com, 22 Oct. 1 room for 3: ¥1,425</t>
+        </is>
+      </c>
+      <c r="N11" s="83" t="inlineStr">
+        <is>
+          <t>Booking.com</t>
         </is>
       </c>
     </row>
@@ -6746,6 +6802,8 @@
       <c r="J12" s="77" t="n"/>
       <c r="K12" s="77" t="n"/>
       <c r="L12" s="77" t="n"/>
+      <c r="M12" s="77" t="n"/>
+      <c r="N12" s="77" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="71" t="inlineStr">
@@ -6801,6 +6859,11 @@
           <t>Tripadvisor→Trip.com, 22 Oct. independent – check photos / foreign guests</t>
         </is>
       </c>
+      <c r="N13" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="71" t="inlineStr">
@@ -6856,6 +6919,11 @@
           <t>Tripadvisor→Agoda, 22 Oct. chain</t>
         </is>
       </c>
+      <c r="N14" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="71" t="inlineStr">
@@ -6911,6 +6979,11 @@
           <t>Tripadvisor→Trip.com, 22 Oct. chain</t>
         </is>
       </c>
+      <c r="N15" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="71" t="inlineStr">
@@ -6966,6 +7039,11 @@
           <t>Tripadvisor→Trip.com (1 room, 3 ppl), 22 Oct. chain</t>
         </is>
       </c>
+      <c r="N16" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="71" t="inlineStr">
@@ -7021,6 +7099,11 @@
           <t>Tripadvisor→Trip.com, 22 Oct. apartment</t>
         </is>
       </c>
+      <c r="N17" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="71" t="inlineStr">
@@ -7076,6 +7159,11 @@
           <t>Tripadvisor→Trip.com, 22 Oct. independent</t>
         </is>
       </c>
+      <c r="N18" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="71" t="inlineStr">
@@ -7131,6 +7219,11 @@
           <t>Tripadvisor→Trip.com, 22 Oct. hostel, private rooms</t>
         </is>
       </c>
+      <c r="N19" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="71" t="inlineStr">
@@ -7186,6 +7279,11 @@
           <t>Tripadvisor→Agoda, 22 Oct. chain</t>
         </is>
       </c>
+      <c r="N20" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="71" t="inlineStr">
@@ -7239,6 +7337,11 @@
       <c r="L21" s="71" t="inlineStr">
         <is>
           <t>Tripadvisor→Trip.com, 22 Oct. chain</t>
+        </is>
+      </c>
+      <c r="N21" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
         </is>
       </c>
     </row>
@@ -7259,6 +7362,8 @@
       <c r="J22" s="77" t="n"/>
       <c r="K22" s="77" t="n"/>
       <c r="L22" s="77" t="n"/>
+      <c r="M22" s="77" t="n"/>
+      <c r="N22" s="77" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="71" t="inlineStr">
@@ -7314,6 +7419,11 @@
           <t>Tripadvisor→Vio, 22 Oct. independent</t>
         </is>
       </c>
+      <c r="N23" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="71" t="inlineStr">
@@ -7369,6 +7479,11 @@
           <t>Tripadvisor→Trip.com, 22 Oct. independent</t>
         </is>
       </c>
+      <c r="N24" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="71" t="inlineStr">
@@ -7424,6 +7539,11 @@
           <t>Tripadvisor→Trip.com, 22 Oct. independent</t>
         </is>
       </c>
+      <c r="N25" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="71" t="inlineStr">
@@ -7479,6 +7599,11 @@
           <t>Tripadvisor→Vio, 22 Oct. chain</t>
         </is>
       </c>
+      <c r="N26" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="71" t="inlineStr">
@@ -7534,6 +7659,11 @@
           <t>Tripadvisor→Trip.com, 22 Oct. chain</t>
         </is>
       </c>
+      <c r="N27" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="71" t="inlineStr">
@@ -7581,12 +7711,22 @@
       </c>
       <c r="K28" s="71" t="inlineStr">
         <is>
-          <t>Booking 7.5 (7); TA 4.7 (3)</t>
+          <t>Trip.com 8.7 (935); Booking 7.5 (7)</t>
         </is>
       </c>
       <c r="L28" s="71" t="inlineStr">
         <is>
-          <t>Tripadvisor→Booking.com, 22 Oct. Booking.com direct ¥516 (2 rooms) / ¥266 (1 room for 3)</t>
+          <t>Tripadvisor→Booking.com, 22 Oct. Booking.com direct ¥516 (2 rooms) / ¥266 (1 room for 3). Reviews: no lift, small rooms</t>
+        </is>
+      </c>
+      <c r="M28" s="83" t="inlineStr">
+        <is>
+          <t>Trip.com</t>
+        </is>
+      </c>
+      <c r="N28" s="83" t="inlineStr">
+        <is>
+          <t>Booking.com</t>
         </is>
       </c>
     </row>
@@ -7644,6 +7784,11 @@
           <t>Tripadvisor→Trip.com, 22 Oct. independent</t>
         </is>
       </c>
+      <c r="N29" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="71" t="inlineStr">
@@ -7699,6 +7844,11 @@
           <t>Tripadvisor→Trip.com, 22 Oct. chain</t>
         </is>
       </c>
+      <c r="N30" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="71" t="inlineStr">
@@ -7754,6 +7904,11 @@
           <t>Tripadvisor→Trip.com, 22 Oct. chain</t>
         </is>
       </c>
+      <c r="N31" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="71" t="inlineStr">
@@ -7809,6 +7964,11 @@
           <t>Tripadvisor→Vio, 22 Oct. chain</t>
         </is>
       </c>
+      <c r="N32" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="71" t="inlineStr">
@@ -7864,6 +8024,11 @@
           <t>Tripadvisor→Priceline, 22 Oct. chain</t>
         </is>
       </c>
+      <c r="N33" s="83" t="inlineStr">
+        <is>
+          <t>Tripadvisor</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="71" t="inlineStr">
@@ -7919,6 +8084,11 @@
           <t>Booking.com, 22 Oct. chain</t>
         </is>
       </c>
+      <c r="N34" s="83" t="inlineStr">
+        <is>
+          <t>Booking.com</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="71" t="inlineStr">
@@ -7974,6 +8144,11 @@
           <t>Tripadvisor→Booking.com, 22 Oct. Booking.com direct ¥906 (2 rooms)</t>
         </is>
       </c>
+      <c r="N35" s="83" t="inlineStr">
+        <is>
+          <t>Booking.com</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="71" t="inlineStr">
@@ -8027,6 +8202,11 @@
       <c r="L36" s="71" t="inlineStr">
         <is>
           <t>Booking.com (1 room, 3 ppl), 22 Oct. chain</t>
+        </is>
+      </c>
+      <c r="N36" s="83" t="inlineStr">
+        <is>
+          <t>Booking.com</t>
         </is>
       </c>
     </row>
@@ -8047,6 +8227,8 @@
       <c r="J37" s="77" t="n"/>
       <c r="K37" s="77" t="n"/>
       <c r="L37" s="77" t="n"/>
+      <c r="M37" s="77" t="n"/>
+      <c r="N37" s="77" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="71" t="inlineStr">
@@ -8060,7 +8242,7 @@
         </is>
       </c>
       <c r="C38" s="71" t="n">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
       <c r="D38" s="71" t="n"/>
       <c r="E38" s="71" t="n"/>
@@ -8080,12 +8262,17 @@
       </c>
       <c r="K38" s="71" t="inlineStr">
         <is>
-          <t>9.8 (957)</t>
+          <t>9.8 (950)</t>
         </is>
       </c>
       <c r="L38" s="71" t="inlineStr">
         <is>
-          <t>Trip.com 1 Oct, 12–15 Nov, 1 room for 4. Cheapest well-rated option; re-check before booking</t>
+          <t>Trip.com 1 Oct, 12–15 Nov, 1 room for 4 (1 queen + 1 futon). 22 Oct page shows 'from USD 78' average, so the ¥528 rate may be gone; accepts foreign guests</t>
+        </is>
+      </c>
+      <c r="M38" s="83" t="inlineStr">
+        <is>
+          <t>Trip.com</t>
         </is>
       </c>
     </row>
@@ -8101,7 +8288,7 @@
         </is>
       </c>
       <c r="C39" s="71" t="n">
-        <v>1.3</v>
+        <v>0.85</v>
       </c>
       <c r="D39" s="71" t="n"/>
       <c r="E39" s="71" t="n"/>
@@ -8121,12 +8308,17 @@
       </c>
       <c r="K39" s="71" t="inlineStr">
         <is>
-          <t>9.6 (1,802)</t>
+          <t>9.5 (1,799)</t>
         </is>
       </c>
       <c r="L39" s="71" t="inlineStr">
         <is>
           <t>Trip.com 1 Oct, 1 room for 3 or 4 (used in Shenyang – Comfort)</t>
+        </is>
+      </c>
+      <c r="M39" s="83" t="inlineStr">
+        <is>
+          <t>Trip.com</t>
         </is>
       </c>
     </row>
@@ -8162,12 +8354,17 @@
       </c>
       <c r="K40" s="71" t="inlineStr">
         <is>
-          <t>9.6</t>
+          <t>9.5 (1,190)</t>
         </is>
       </c>
       <c r="L40" s="71" t="inlineStr">
         <is>
-          <t>Trip.com 22 Oct; same hotel as Jin Ke above</t>
+          <t>Trip.com 22 Oct; same hotel as Jin Ke above (19 Wenhua Road)</t>
+        </is>
+      </c>
+      <c r="M40" s="83" t="inlineStr">
+        <is>
+          <t>Trip.com</t>
         </is>
       </c>
     </row>
@@ -8182,7 +8379,9 @@
           <t>Birches Hotel – 2 rooms (double beds, windowless)</t>
         </is>
       </c>
-      <c r="C41" s="71" t="n"/>
+      <c r="C41" s="71" t="n">
+        <v>0.79</v>
+      </c>
       <c r="D41" s="71" t="n"/>
       <c r="E41" s="71" t="n"/>
       <c r="F41" s="71" t="n"/>
@@ -8201,12 +8400,17 @@
       </c>
       <c r="K41" s="71" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>9.2 (1,377)</t>
         </is>
       </c>
       <c r="L41" s="71" t="inlineStr">
         <is>
           <t>Trip.com 22 Oct</t>
+        </is>
+      </c>
+      <c r="M41" s="83" t="inlineStr">
+        <is>
+          <t>Trip.com</t>
         </is>
       </c>
     </row>
@@ -8222,7 +8426,7 @@
         </is>
       </c>
       <c r="C42" s="71" t="n">
-        <v>1.3</v>
+        <v>0.85</v>
       </c>
       <c r="D42" s="71" t="n"/>
       <c r="E42" s="71" t="n"/>
@@ -8242,12 +8446,17 @@
       </c>
       <c r="K42" s="71" t="inlineStr">
         <is>
-          <t>9.5</t>
+          <t>9.5 (1,799)</t>
         </is>
       </c>
       <c r="L42" s="71" t="inlineStr">
         <is>
           <t>Trip.com 22 Oct</t>
+        </is>
+      </c>
+      <c r="M42" s="83" t="inlineStr">
+        <is>
+          <t>Trip.com</t>
         </is>
       </c>
     </row>
@@ -8283,12 +8492,17 @@
       </c>
       <c r="K43" s="71" t="inlineStr">
         <is>
-          <t>9.0 (1,433)</t>
+          <t>9.3 (1,663)</t>
         </is>
       </c>
       <c r="L43" s="71" t="inlineStr">
         <is>
-          <t>Trip.com 22 Oct; twin beds (used in Shenyang – Sleep value)</t>
+          <t>Trip.com 22 Oct; twin beds, 55 Sanhao Street (used in Shenyang – Sleep value)</t>
+        </is>
+      </c>
+      <c r="M43" s="83" t="inlineStr">
+        <is>
+          <t>Trip.com</t>
         </is>
       </c>
     </row>
@@ -8343,7 +8557,7 @@
         </is>
       </c>
       <c r="C45" s="71" t="n">
-        <v>0.58</v>
+        <v>0.54</v>
       </c>
       <c r="D45" s="71" t="n"/>
       <c r="E45" s="71" t="n"/>
@@ -8363,12 +8577,17 @@
       </c>
       <c r="K45" s="71" t="inlineStr">
         <is>
-          <t>9.7 (1,998)</t>
+          <t>9.7 (1,997)</t>
         </is>
       </c>
       <c r="L45" s="71" t="inlineStr">
         <is>
           <t>Trip.com 22 Oct, 30% 'Surprise Savings' rate (used in Shenyang – Sleep first)</t>
+        </is>
+      </c>
+      <c r="M45" s="83" t="inlineStr">
+        <is>
+          <t>Trip.com</t>
         </is>
       </c>
     </row>
@@ -8404,12 +8623,17 @@
       </c>
       <c r="K46" s="71" t="inlineStr">
         <is>
-          <t>8.2 (1,062)</t>
+          <t>8.7 (935)</t>
         </is>
       </c>
       <c r="L46" s="71" t="inlineStr">
         <is>
-          <t>Trip.com 1 Oct, 13–15 Nov; Booking.com 22 Oct ¥516 for 3 nights</t>
+          <t>Trip.com 1 Oct, 13–15 Nov; Booking.com 22 Oct ¥516 for 3 nights. No lift, small rooms (reviews)</t>
+        </is>
+      </c>
+      <c r="M46" s="83" t="inlineStr">
+        <is>
+          <t>Trip.com</t>
         </is>
       </c>
     </row>
@@ -8777,12 +9001,53 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A52:L52"/>
-    <mergeCell ref="A51:L51"/>
-    <mergeCell ref="A49:L49"/>
-    <mergeCell ref="A50:L50"/>
+    <mergeCell ref="A50:N50"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A52:N52"/>
+    <mergeCell ref="A51:N51"/>
+    <mergeCell ref="A49:N49"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N32" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N35" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N36" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId39"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>